<commit_message>
employe portal has been updated
</commit_message>
<xml_diff>
--- a/attendance/python-script/all_users_commercial_branch.xlsx
+++ b/attendance/python-script/all_users_commercial_branch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2711,6 +2711,33 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>5079</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Vaiz</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chat module issue has been fixed
</commit_message>
<xml_diff>
--- a/attendance/python-script/all_users_commercial_branch.xlsx
+++ b/attendance/python-script/all_users_commercial_branch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2738,6 +2738,195 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>5080</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Hammad.Haroon</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>5081</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Asad.Ali</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>5082</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Gohar.Anil</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>5083</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Surriya.Rehman</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>5084</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Adan</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>5085</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Abdul.Wasi</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>5086</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Aftab.Ahmad</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
salary broadcast  has been updated
</commit_message>
<xml_diff>
--- a/attendance/python-script/all_users_commercial_branch.xlsx
+++ b/attendance/python-script/all_users_commercial_branch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E145"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,12 +608,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5001</t>
+          <t>4041</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Owais</t>
+          <t>Bakhtawar.Mehmood</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5002</t>
+          <t>5001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abdulhadi</t>
+          <t>Owais</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -662,12 +662,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5003</t>
+          <t>5002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hamza</t>
+          <t>Abdulhadi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -689,12 +689,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5004</t>
+          <t>5003</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Faizan</t>
+          <t>Hamza</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5005</t>
+          <t>5004</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Haris</t>
+          <t>Faizan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -743,12 +743,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5006</t>
+          <t>5005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ali</t>
+          <t>Haris</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -770,12 +770,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5007</t>
+          <t>5006</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Noroz</t>
+          <t>Ali</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5008</t>
+          <t>5007</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hizbullah</t>
+          <t>Noroz</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -824,12 +824,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5009</t>
+          <t>5008</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Hasnain</t>
+          <t>Hizbullah</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -851,12 +851,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5010</t>
+          <t>5009</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Furqan</t>
+          <t>Hasnain</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -878,12 +878,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5010</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Basit</t>
+          <t>Furqan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -905,12 +905,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5012</t>
+          <t>5011</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Romis</t>
+          <t>Basit</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -932,12 +932,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5013</t>
+          <t>5012</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Romis</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -959,12 +959,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5014</t>
+          <t>5013</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Moaznaeem</t>
+          <t>David</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -986,12 +986,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5015</t>
+          <t>5014</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Muneeb</t>
+          <t>Moaznaeem</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1013,12 +1013,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5016</t>
+          <t>5015</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Khalil</t>
+          <t>Muneeb</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1040,12 +1040,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5017</t>
+          <t>5016</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ahsan</t>
+          <t>Khalil</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5018</t>
+          <t>5017</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Fardad</t>
+          <t>Ahsan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1094,12 +1094,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5019</t>
+          <t>5018</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Sikandar</t>
+          <t>Fardad</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1121,12 +1121,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5020</t>
+          <t>5019</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aqeel</t>
+          <t>Sikandar</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1148,12 +1148,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>5020</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Shumaz</t>
+          <t>Aqeel</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1175,12 +1175,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5022</t>
+          <t>5021</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Huzaifa</t>
+          <t>Shumaz</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1202,12 +1202,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5023</t>
+          <t>5022</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Moiz</t>
+          <t>Huzaifa</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1229,12 +1229,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5024</t>
+          <t>5023</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Arzo</t>
+          <t>Moiz</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1256,12 +1256,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>5024</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Asima</t>
+          <t>Arzo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1283,12 +1283,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5026</t>
+          <t>5025</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Shamsulhaq</t>
+          <t>Asima</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1310,12 +1310,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t>5026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Faisal</t>
+          <t>Shamsulhaq</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1337,12 +1337,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5028</t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Muhammadali</t>
+          <t>Faisal</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1364,12 +1364,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5029</t>
+          <t>5028</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Abubaker</t>
+          <t>Muhammadali</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1391,12 +1391,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>5029</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Zeshan</t>
+          <t>Abubaker</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1418,12 +1418,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5031</t>
+          <t>5030</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Tayelamjad</t>
+          <t>Zeshan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1445,12 +1445,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5032</t>
+          <t>5031</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Haseebhaider</t>
+          <t>Tayelamjad</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1472,12 +1472,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5033</t>
+          <t>5032</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Maneeque</t>
+          <t>Haseebhaider</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1499,12 +1499,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>5033</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Awaisatti</t>
+          <t>Maneeque</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1526,12 +1526,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5035</t>
+          <t>5034</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alishaali</t>
+          <t>Awaisatti</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1553,12 +1553,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5036</t>
+          <t>5035</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Javeriali</t>
+          <t>Alishaali</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1580,12 +1580,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>5037</t>
+          <t>5036</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Farhanmalik</t>
+          <t>Javeriali</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1607,12 +1607,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>5038</t>
+          <t>5037</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Hashim</t>
+          <t>Farhanmalik</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1634,12 +1634,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5039</t>
+          <t>5038</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Raheel</t>
+          <t>Hashim</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1661,12 +1661,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5040</t>
+          <t>5039</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Mkamal</t>
+          <t>Raheel</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1688,12 +1688,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5040</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Rajaobaidullah</t>
+          <t>Mkamal</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1715,12 +1715,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>5041</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Azharhussain</t>
+          <t>Rajaobaidullah</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1742,12 +1742,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>5043</t>
+          <t>5042</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Samiullaha</t>
+          <t>Azharhussain</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1769,12 +1769,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>5044</t>
+          <t>5043</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Salman</t>
+          <t>Samiullaha</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1796,12 +1796,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>5045</t>
+          <t>5044</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>mohsin</t>
+          <t>Salman</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1823,12 +1823,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>5046</t>
+          <t>5045</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Kanwal</t>
+          <t>mohsin</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1850,12 +1850,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>5047</t>
+          <t>5046</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Chaudarymuhammadshehryar</t>
+          <t>Kanwal</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1877,12 +1877,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>5047</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Daud</t>
+          <t>Chaudarymuhammadshehryar</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1904,12 +1904,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>5049</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Umershehzad</t>
+          <t>Daud</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1931,12 +1931,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>5050</t>
+          <t>5049</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Altafhussain</t>
+          <t>Umershehzad</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1958,12 +1958,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>5051</t>
+          <t>5050</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Sadamshah</t>
+          <t>Altafhussain</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1985,12 +1985,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>5052</t>
+          <t>5051</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Hammad</t>
+          <t>Sadamshah</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2012,12 +2012,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>5053</t>
+          <t>5052</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Mshabbir</t>
+          <t>Hammad</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2039,12 +2039,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>5054</t>
+          <t>5053</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Uzair</t>
+          <t>Mshabbir</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2066,12 +2066,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>5055</t>
+          <t>5054</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tahir</t>
+          <t>Uzair</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2093,12 +2093,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>5056</t>
+          <t>5055</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Mehmood</t>
+          <t>Tahir</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2120,12 +2120,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>5057</t>
+          <t>5056</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Hashmi</t>
+          <t>Mehmood</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2147,12 +2147,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>5058</t>
+          <t>5057</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Mhammad</t>
+          <t>Hashmi</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2174,12 +2174,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>5059</t>
+          <t>5058</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Malikarslan</t>
+          <t>Mhammad</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2201,12 +2201,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>5060</t>
+          <t>5059</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Salmanwaheed</t>
+          <t>Malikarslan</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2228,12 +2228,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>5061</t>
+          <t>5060</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Malikhassan</t>
+          <t>Salmanwaheed</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2255,12 +2255,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>5062</t>
+          <t>5061</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Muskanarif</t>
+          <t>Malikhassan</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2282,12 +2282,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>5063</t>
+          <t>5062</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Abdulwahid</t>
+          <t>Muskanarif</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2309,12 +2309,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>5064</t>
+          <t>5063</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Asadbilal</t>
+          <t>Abdulwahid</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2336,12 +2336,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>5065</t>
+          <t>5064</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Nomanashraf</t>
+          <t>Asadbilal</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2363,12 +2363,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>5066</t>
+          <t>5065</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Mabdullah</t>
+          <t>Nomanashraf</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2390,12 +2390,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>5067</t>
+          <t>5066</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Awaisurrehman</t>
+          <t>Mabdullah</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2417,12 +2417,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>5068</t>
+          <t>5067</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Arbaz</t>
+          <t>Awaisurrehman</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2444,12 +2444,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>5069</t>
+          <t>5068</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Ahsanhassan</t>
+          <t>Arbaz</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2471,17 +2471,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>5070</t>
+          <t>5069</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Syedramish</t>
+          <t>Ahsanhassan</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>User</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2498,17 +2498,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>5071</t>
+          <t>5070</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Misbah</t>
+          <t>Syedramish</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2525,12 +2525,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>5072</t>
+          <t>5071</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Asad</t>
+          <t>Misbah</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2552,12 +2552,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>5073</t>
+          <t>5072</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Rafia</t>
+          <t>Asad</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2579,12 +2579,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>5074</t>
+          <t>5073</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Shazil</t>
+          <t>Rafia</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2606,12 +2606,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>5075</t>
+          <t>5074</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Shehryar</t>
+          <t>Shazil</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2633,12 +2633,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>5076</t>
+          <t>5075</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Hammadakhtar</t>
+          <t>Shehryar</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2660,12 +2660,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>5077</t>
+          <t>5076</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Aliyan</t>
+          <t>Hammadakhtar</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2687,12 +2687,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>5078</t>
+          <t>5077</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MehrabAli</t>
+          <t>Aliyan</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2714,12 +2714,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>5079</t>
+          <t>5078</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Vaiz</t>
+          <t>MehrabAli</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2741,12 +2741,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>5080</t>
+          <t>5079</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Hammad.Haroon</t>
+          <t>Vaiz</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2768,12 +2768,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>5081</t>
+          <t>5080</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Asad.Ali</t>
+          <t>Hammad.Haroon</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2795,12 +2795,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>5082</t>
+          <t>5081</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Gohar.Anil</t>
+          <t>Asad.Ali</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2822,12 +2822,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>5083</t>
+          <t>5082</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Surriya.Rehman</t>
+          <t>Gohar.Anil</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2849,12 +2849,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>5084</t>
+          <t>5083</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Adan</t>
+          <t>Surriya.Rehman</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2876,12 +2876,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>5085</t>
+          <t>5084</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Abdul.Wasi</t>
+          <t>Adan</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2903,12 +2903,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>5086</t>
+          <t>5085</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Aftab.Ahmad</t>
+          <t>Abdul.Wasi</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2930,12 +2930,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>5087</t>
+          <t>5086</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Syeda.Hijab</t>
+          <t>Aftab.Ahmad</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2957,12 +2957,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>5088</t>
+          <t>5087</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CMBilal</t>
+          <t>Syeda.Hijab</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2984,12 +2984,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>5089</t>
+          <t>5088</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>M.Khizar</t>
+          <t>CMBilal</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3011,12 +3011,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>5090</t>
+          <t>5089</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Talha.Chauhan</t>
+          <t>M.Khizar</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3038,12 +3038,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>5091</t>
+          <t>5090</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Saira.Zafar</t>
+          <t>Talha.Chauhan</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3065,12 +3065,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>5092</t>
+          <t>5091</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Araiz</t>
+          <t>Saira.Zafar</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3092,12 +3092,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>5093</t>
+          <t>5092</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Syed.Bilal.Ahmad</t>
+          <t>Araiz</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3119,12 +3119,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>5094</t>
+          <t>5093</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Zeeshan.jan</t>
+          <t>Syed.Bilal.Ahmad</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3146,12 +3146,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>5095</t>
+          <t>5094</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sikandar.Ali</t>
+          <t>Zeeshan.jan</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3173,12 +3173,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>5096</t>
+          <t>5095</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Amir</t>
+          <t>Sikandar.Ali</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -3200,12 +3200,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>5097</t>
+          <t>5096</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>M.Siddique</t>
+          <t>Amir</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3227,12 +3227,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>5098</t>
+          <t>5097</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Hussna</t>
+          <t>M.Siddique</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3254,12 +3254,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>5099</t>
+          <t>5098</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Ameer.Hamza</t>
+          <t>Hussna</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3281,12 +3281,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>5099</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Shaven.Gill</t>
+          <t>Ameer.Hamza</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3308,12 +3308,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Misbah.Mehrban</t>
+          <t>Shaven.Gill</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3335,12 +3335,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>6001</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Amir.nazeer</t>
+          <t>Misbah.Mehrban</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3362,12 +3362,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>6002</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Ejaz</t>
+          <t>Amir.nazeer</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3389,12 +3389,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>6003</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Ahmed.Ali</t>
+          <t>Ejaz</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3416,12 +3416,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>6005</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Zunair</t>
+          <t>Ahmed.Ali</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3443,12 +3443,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>6006</t>
+          <t>6005</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Kiran</t>
+          <t>Zunair</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3470,12 +3470,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>6007</t>
+          <t>6006</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Zeeshan.Abbasi</t>
+          <t>Kiran</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3497,12 +3497,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>6007</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Fahad.Mughal</t>
+          <t>Zeeshan.Abbasi</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3524,12 +3524,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>6009</t>
+          <t>6008</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Abdul.Moeez</t>
+          <t>Fahad.Mughal</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3551,12 +3551,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>6010</t>
+          <t>6009</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Hanook</t>
+          <t>Abdul.Moeez</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3578,12 +3578,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>6010</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Noor</t>
+          <t>Hanook</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3605,12 +3605,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>6012</t>
+          <t>6011</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Maryam</t>
+          <t>Noor</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3632,12 +3632,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>6013</t>
+          <t>6012</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sana.Naz</t>
+          <t>Maryam</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3659,12 +3659,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>6014</t>
+          <t>6013</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Mahaz.Ali</t>
+          <t>Sana.Naz</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3686,12 +3686,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>6015</t>
+          <t>6014</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Abdul.Wahab</t>
+          <t>Mahaz.Ali</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3713,12 +3713,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>6016</t>
+          <t>6015</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Rayyan</t>
+          <t>Abdul.Wahab</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3740,12 +3740,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>6016</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Mudassar.Khan</t>
+          <t>Rayyan</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3767,12 +3767,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>6018</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Hannah</t>
+          <t>Mudassar.Khan</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3794,12 +3794,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>6019</t>
+          <t>6018</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Adeel.Afzal</t>
+          <t>Hannah</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3821,12 +3821,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>6020</t>
+          <t>6019</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Ali.Shah</t>
+          <t>Adeel.Afzal</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3848,12 +3848,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>6020</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Bilal.Hanif</t>
+          <t>Ali.Shah</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3875,12 +3875,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>6022</t>
+          <t>6021</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Hasnain</t>
+          <t>Bilal.Hanif</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3902,12 +3902,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>6023</t>
+          <t>6022</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Kabeer</t>
+          <t>Hasnain</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3929,12 +3929,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>6024</t>
+          <t>6023</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Sarmad</t>
+          <t>Kabeer</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3956,12 +3956,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>6024</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>M.Asad</t>
+          <t>Sarmad</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3983,12 +3983,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>6026</t>
+          <t>6025</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Mueed</t>
+          <t>M.Asad</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4010,12 +4010,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>6026</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Atif</t>
+          <t>Mueed</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -4037,12 +4037,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>6027</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Raja.Haider</t>
+          <t>Atif</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -4064,12 +4064,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>6028</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Mohid.Hadi</t>
+          <t>Raja.Haider</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -4091,12 +4091,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>6030</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Mazhar</t>
+          <t>Mohid.Hadi</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4118,12 +4118,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>6031</t>
+          <t>6030</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Naila.Raja</t>
+          <t>Mazhar</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -4145,12 +4145,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>6032</t>
+          <t>6031</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Rimsha</t>
+          <t>Naila.Raja</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -4172,12 +4172,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>6033</t>
+          <t>6032</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Farhana</t>
+          <t>Rimsha</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -4199,12 +4199,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>6034</t>
+          <t>6033</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Rubab</t>
+          <t>Farhana</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -4226,12 +4226,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>6035</t>
+          <t>6034</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Momina</t>
+          <t>Rubab</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4253,12 +4253,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>6036</t>
+          <t>6035</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Nayab.Naveed</t>
+          <t>Momina</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -4280,12 +4280,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>6037</t>
+          <t>6036</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Jibran.Khan</t>
+          <t>Nayab.Naveed</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -4307,25 +4307,295 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
+          <t>6037</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Jibran.Khan</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
           <t>6038</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
+      <c r="B146" t="inlineStr">
         <is>
           <t>Naseer.Hussain</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Commercial Branch</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>6039</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Malik.Shujah</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>6040</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Tahir.younas</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>6042</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>M.Abdullah</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>6043</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Mohsin.Zahid</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>6044</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Areez</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>6045</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Syed.Shabab</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>6046</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Ali.Imran</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>6047</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Ammar.Hassan</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>6048</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Rana.Shoaib</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
         <is>
           <t>125.209.68.118</t>
         </is>

</xml_diff>

<commit_message>
workfromhome portal has been developed
</commit_message>
<xml_diff>
--- a/attendance/python-script/all_users_commercial_branch.xlsx
+++ b/attendance/python-script/all_users_commercial_branch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E158"/>
+  <dimension ref="A1:E168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4682,6 +4682,276 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>6052</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Syed.Imran</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>6053</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Hasan</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>6054</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Mehreen.Butt</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>6055</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Abubakr.Siddique</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>6056</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Ashir</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>6057</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Abdullah,Almas</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>6058</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Usman,Yousuf</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>6059</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Aiza.Baig</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>6060</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Abdul.Wasay</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>6061</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Suleman.Yasir</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Commercial Branch</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>125.209.68.118</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>